<commit_message>
Added TC01 - Normal Plan - Single Lab request - Account
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData_Trail.xlsx
+++ b/src/main/resources/TestData_Trail.xlsx
@@ -528,7 +528,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:G66"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -656,9 +656,855 @@
         <v>harish@tester2.com</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B25" t="str">
+        <v>PlanType</v>
+      </c>
+      <c r="C25" t="str">
+        <v>LabRequestType</v>
+      </c>
+      <c r="D25" t="str">
+        <v>LabType</v>
+      </c>
+      <c r="E25" t="str">
+        <v>TeamName</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PlanId</v>
+      </c>
+      <c r="G25" t="str">
+        <v>RunFlag_x000d_</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC01</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Account</v>
+      </c>
+      <c r="E26" t="str">
+        <v>harish</v>
+      </c>
+      <c r="F26" t="str">
+        <v>1365</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC02</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Region based plan</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Region based plan</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Single Lab request</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC26</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Cohort lab</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC27</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC28</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC29</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Normal Plan</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC30</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC31</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC32</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Plan with expiry date</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC33</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC34</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC35</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Plan with default policy</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC36</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC37</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC38</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Plan with configured duration</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Batch provision</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC39</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Account</v>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC40</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Deployment</v>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v>Y_x000d_</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC41</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Lazy Lab request</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Composition</v>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+      <c r="G66" t="str">
+        <v>Y</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
single and cohort lab request code
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData_Trail.xlsx
+++ b/src/main/resources/TestData_Trail.xlsx
@@ -528,7 +528,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:H66"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -678,6 +678,9 @@
       <c r="G25" t="str">
         <v>RunFlag_x000d_</v>
       </c>
+      <c r="H25" t="str">
+        <v>extra data</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -755,8 +758,11 @@
       <c r="D29" t="str">
         <v>Account</v>
       </c>
+      <c r="E29" t="str">
+        <v>harish</v>
+      </c>
       <c r="F29" t="str">
-        <v/>
+        <v>1371</v>
       </c>
       <c r="G29" t="str">
         <v>Y_x000d_</v>
@@ -815,11 +821,17 @@
       <c r="D32" t="str">
         <v>Account</v>
       </c>
+      <c r="E32" t="str">
+        <v>harish</v>
+      </c>
       <c r="F32" t="str">
-        <v/>
+        <v>1371</v>
       </c>
       <c r="G32" t="str">
         <v>Y_x000d_</v>
+      </c>
+      <c r="H32" t="str">
+        <v>NotifyBefore1Day</v>
       </c>
     </row>
     <row r="33">
@@ -875,8 +887,11 @@
       <c r="D35" t="str">
         <v>Account</v>
       </c>
+      <c r="E35" t="str">
+        <v>harish</v>
+      </c>
       <c r="F35" t="str">
-        <v/>
+        <v>1373</v>
       </c>
       <c r="G35" t="str">
         <v>Y_x000d_</v>
@@ -975,8 +990,11 @@
       <c r="D40" t="str">
         <v>Account</v>
       </c>
+      <c r="E40" t="str">
+        <v>harish</v>
+      </c>
       <c r="F40" t="str">
-        <v/>
+        <v>1369</v>
       </c>
       <c r="G40" t="str">
         <v>Y_x000d_</v>
@@ -1035,8 +1053,11 @@
       <c r="D43" t="str">
         <v>Account</v>
       </c>
+      <c r="E43" t="str">
+        <v>harish</v>
+      </c>
       <c r="F43" t="str">
-        <v/>
+        <v>1372</v>
       </c>
       <c r="G43" t="str">
         <v>Y_x000d_</v>
@@ -1095,11 +1116,17 @@
       <c r="D46" t="str">
         <v>Account</v>
       </c>
+      <c r="E46" t="str">
+        <v>harish</v>
+      </c>
       <c r="F46" t="str">
-        <v/>
+        <v>1372</v>
       </c>
       <c r="G46" t="str">
         <v>Y_x000d_</v>
+      </c>
+      <c r="H46" t="str">
+        <v>NotifyBefore1Day</v>
       </c>
     </row>
     <row r="47">
@@ -1155,8 +1182,11 @@
       <c r="D49" t="str">
         <v>Account</v>
       </c>
+      <c r="E49" t="str">
+        <v>harish</v>
+      </c>
       <c r="F49" t="str">
-        <v/>
+        <v>1374</v>
       </c>
       <c r="G49" t="str">
         <v>Y_x000d_</v>
@@ -1504,7 +1534,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>